<commit_message>
Refresh sample data and simplify Excel export.
Use a four-row sales_example.xlsx, add grouped-by-product links on the upload page, and export only the Summary sheet. Lock sample totals with a regression test.
</commit_message>
<xml_diff>
--- a/examples/sales_example.xlsx
+++ b/examples/sales_example.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,21 +425,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Region</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
@@ -456,11 +468,41 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C3" t="n">
         <v>25</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>